<commit_message>
Make training workbook import tolerant of an offset header row
MS-NID.xlsx had a title row above its real "SL NO | Request | Reply"
header, which made xlsx's sheet_to_json synthesize __EMPTY column
names from row 1 and silently drop every data row as unparseable —
0 examples extracted even after the workbook was updated with real
content.

readWorkbook now reads each sheet as a raw array-of-arrays first and
scans the first 10 rows for one containing a recognized Request/Reply
header label, instead of assuming row 1 is always the header. Falls
back to row 1 if no header is found, so well-formed workbooks (the
other 4 curated files) are unaffected.

User also fixed the workbook's layout directly (deleted the extra
leading row) — both fixes land together since either alone only
partially explains the original 0-example bug.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Training Data/Automation/MS-NID.xlsx
+++ b/Training Data/Automation/MS-NID.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\GitHub\SMS_Automation\Training Data\Automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Documents\GitHub\SMS_Automation\Training Data\Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B0D9248-1BD8-40B8-8EE2-131565EC2EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF0D113B-D08E-4F6C-9254-07A02C1E14B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MS-NID" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>Request</t>
   </si>
@@ -100,13 +100,50 @@
     <t>MSISDN?8801990169712 national_id?
 Document Number?19790619431282189?
 Date of Birth?1979-01-01</t>
+  </si>
+  <si>
+    <t>MS-NID 01881986611</t>
+  </si>
+  <si>
+    <t>MSISDN: 8801881986611
+NID: 2854786395
+DoB: 11/03/1996 [Robi]</t>
+  </si>
+  <si>
+    <t>MS-NID 01600204240</t>
+  </si>
+  <si>
+    <t>MS-NID 01603990945</t>
+  </si>
+  <si>
+    <t>MSISDN: 8801603990945
+NID: 3769269055
+DoB: 12/20/2003 [Robi]</t>
+  </si>
+  <si>
+    <t>MSISDN: 8801600204240
+NID: 5561211730
+DoB: 01/07/2001 [Robi]</t>
+  </si>
+  <si>
+    <t>01904809964 NID 19912610457000031  DOB 10.12.1991</t>
+  </si>
+  <si>
+    <t>MS-NID 01603990946</t>
+  </si>
+  <si>
+    <t>MS-NID 01938590648</t>
+  </si>
+  <si>
+    <t>MSISDN?8801938590648 NID 5108405506?
+Date of Birth?2001-01-12</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -619,13 +656,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -700,7 +737,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0247DF39-8DB6-46DB-A503-184C0D447B03}" name="Table1" displayName="Table1" ref="B2:C16" headerRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0247DF39-8DB6-46DB-A503-184C0D447B03}" name="Table1" displayName="Table1" ref="B1:C17" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="2">
     <tableColumn id="2" xr3:uid="{7D16482E-AEB6-40B8-AF25-B22E6FAE885B}" name="Column2" headerRowDxfId="3" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{B92D272C-C50B-4A58-8D48-62AA928425A5}" name="Column3" headerRowDxfId="1" dataDxfId="0"/>
@@ -1026,163 +1063,214 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" style="1"/>
-    <col min="2" max="2" width="23.31640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="86.81640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.75" style="1"/>
+    <col min="2" max="2" width="23.375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="86.875" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="B1"/>
-      <c r="C1"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A2" s="4" t="s">
+    <row r="1" spans="1:3">
+      <c r="A1" s="4" t="s">
         <v>20</v>
       </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="6">
+        <v>1</v>
+      </c>
       <c r="B2" s="2" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A3" s="6">
-        <v>1</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="4">
+        <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A4" s="4">
-        <v>3</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="5">
+        <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A5" s="5">
-        <v>4</v>
-      </c>
       <c r="B5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="5">
         <v>6</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="B6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="4">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A6" s="4">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="B7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="5">
         <v>8</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="B8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="4">
         <v>9</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A7" s="5">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="B9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="28.5">
+      <c r="A10" s="5">
         <v>10</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="B10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="42.75">
+      <c r="A11" s="4">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A8" s="4">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="s">
+      <c r="B11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="42.75">
+      <c r="A12" s="5">
         <v>12</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="B12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="42.75">
+      <c r="A13" s="4">
         <v>13</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A9" s="5">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="s">
+      <c r="B13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="42.75">
+      <c r="A14" s="5">
         <v>14</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="B14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="42.75">
+      <c r="A15" s="4">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A10" s="4">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="s">
+      <c r="B15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="4">
         <v>16</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="B16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="28.5">
+      <c r="A17" s="5">
         <v>17</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="29.5" x14ac:dyDescent="0.75">
-      <c r="A11" s="5">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="s">
+      <c r="B17" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="4">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="4">
         <v>19</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
-      <c r="A12" s="4">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="44.25" x14ac:dyDescent="0.75">
-      <c r="A13" s="5">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A14" s="4">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A15" s="5">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A16" s="4">
-        <v>15</v>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="5">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>